<commit_message>
Test calculation of volume from mass
</commit_message>
<xml_diff>
--- a/tests/data/applications/Source_Plate.xlsx
+++ b/tests/data/applications/Source_Plate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="content" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="20">
   <si>
     <t xml:space="preserve">A</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WATER</t>
   </si>
 </sst>
 </file>
@@ -202,7 +205,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Y93"/>
-  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.12"/>
@@ -724,7 +727,9 @@
       <c r="V17" s="3"/>
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
-      <c r="Y17" s="3"/>
+      <c r="Y17" s="3" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -819,7 +824,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Y19"/>
-  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="n">
@@ -2124,7 +2129,7 @@
         <v>0</v>
       </c>
       <c r="Y17" s="3" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2146,7 +2151,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultColWidth="8.578125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.60546875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="n">
@@ -2304,7 +2309,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="0" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="0" t="n">
         <v>0</v>
@@ -3451,7 +3456,7 @@
         <v>0</v>
       </c>
       <c r="Y17" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>